<commit_message>
Arsip: perbaiki username kosong + kelola dokumen (ubah/arsipkan/hapus)
</commit_message>
<xml_diff>
--- a/backend/Database-Arsip-LSP-UNIMED.xlsx
+++ b/backend/Database-Arsip-LSP-UNIMED.xlsx
@@ -558,7 +558,6 @@
           <t>2026-10-05T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>072/LSP-UNIMED/SK/X/2026</t>
@@ -584,7 +583,6 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Disahkan</t>
@@ -613,9 +611,6 @@
           <t>{"tanggal":"2026-10-05"}</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -628,7 +623,6 @@
           <t>2026-10-09T00:00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>074/LSP-UNIMED/UND/X/2026</t>
@@ -654,7 +648,6 @@
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Draf</t>
@@ -683,9 +676,6 @@
           <t>{"tanggal":"2026-10-09","tglAcara":"2026-10-20"}</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -698,7 +688,6 @@
           <t>2026-09-30T00:00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>LSP-UNIMED/MUT/005/2026</t>
@@ -724,7 +713,6 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Berlaku</t>
@@ -733,17 +721,11 @@
       <c r="K4" t="n">
         <v>9</v>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>Daftar_Induk_Dokumen.pdf</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:R1"/>
@@ -771,48 +753,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="22" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>dibuat</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>diubah</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>nama</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>peran</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>salt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>password_hash</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>aktif</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>bagian</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>email</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>aktif</t>
         </is>
       </c>
     </row>
@@ -822,23 +819,26 @@
           <t>u000000001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
+          <t>ketua</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Ketua LSP</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Ketua LSP</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>YA</t>
         </is>
       </c>
     </row>
@@ -848,23 +848,26 @@
           <t>u000000002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Admin Arsip</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>YA</t>
         </is>
       </c>
     </row>
@@ -874,27 +877,31 @@
           <t>u000000003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
+          <t>sekretariat</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>YA</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Sekretariat</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -904,27 +911,31 @@
           <t>u000000004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
+          <t>sertifikasi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Bidang Sertifikasi</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Bidang Sertifikasi</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>YA</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Bidang Sertifikasi</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -934,27 +945,31 @@
           <t>u000000005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
+          <t>mutu</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Manajemen Mutu</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Manajemen Mutu</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>YA</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Manajemen Mutu</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -964,27 +979,31 @@
           <t>u000000006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
+          <t>skema</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Bidang Skema</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Bidang Skema</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>YA</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Bidang Skema</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -994,27 +1013,31 @@
           <t>u000000007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
+          <t>administrasi</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Administrasi</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Administrasi</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>YA</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Administrasi</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1107,6 @@
           <t>2026-10-09T15:42:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>2026-10-09 15:42</t>
@@ -1240,7 +1262,6 @@
           <t>2026-10-09T15:42:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>d000000003</t>
@@ -1264,7 +1285,6 @@
           <t>Revisi 9 Daftar Induk Dokumen</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -1354,7 +1374,6 @@
           <t>2026-09-20T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>SM-040/2026</t>
@@ -1395,7 +1414,6 @@
           <t>Didisposisi</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1408,7 +1426,6 @@
           <t>2026-10-08T00:00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>SM-043/2026</t>
@@ -1449,7 +1466,6 @@
           <t>Diterima</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
@@ -1537,7 +1553,6 @@
           <t>2026-09-20T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>s000000001</t>
@@ -1568,7 +1583,6 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -1648,7 +1662,6 @@
           <t>2026-10-05T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>072/LSP-UNIMED/SK/X/2026</t>
@@ -1677,7 +1690,6 @@
           <t>d000000001</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1690,7 +1702,6 @@
           <t>2026-10-09T00:00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>074/LSP-UNIMED/UND/X/2026</t>
@@ -1719,7 +1730,6 @@
           <t>d000000002</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -1784,7 +1794,6 @@
           <t>2026-10-10T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Penyaksian (witness) uji kompetensi BNSP</t>
@@ -1817,7 +1826,6 @@
           <t>2026-10-10T00:00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Rapat pleno hasil uji kompetensi</t>
@@ -1902,7 +1910,6 @@
           <t>2026-10-10T00:00:00</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>a000000001</t>
@@ -1935,7 +1942,6 @@
           <t>2026-10-10T00:00:00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>a000000001</t>
@@ -1968,7 +1974,6 @@
           <t>2026-10-10T00:00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>a000000002</t>
@@ -2053,8 +2058,6 @@
           <t>t000000001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>undangan</t>
@@ -2082,8 +2085,6 @@
           <t>t000000002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>tugas</t>
@@ -2111,8 +2112,6 @@
           <t>t000000003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>sk</t>
@@ -2140,8 +2139,6 @@
           <t>t000000004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>ba</t>
@@ -2169,8 +2166,6 @@
           <t>t000000005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>hadir</t>
@@ -2198,8 +2193,6 @@
           <t>t000000006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>notulen</t>
@@ -2304,8 +2297,6 @@
           <t>k000000001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>LEMBAGA SERTIFIKASI PROFESI</t>

</xml_diff>